<commit_message>
Add AirSourceHeatPumpHeating class for hot water (heating) mode
- AirSourceHeatPump（冷房専用）と対称な温水モード専用クラスを追加（既存クラスは無変更）
- equipment_spec.xlsx に AirSourceHeatPumpHeating シートを追加（外気温 -15~15C x 負荷率 0.2~1.0 のCOP表サンプル、既存シートは無変更）
- COPは表補間 + 暖房カルノー効率比による温水出口温度補正（補正係数上限2.0）

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/equipment_spec.xlsx
+++ b/equipment_spec.xlsx
@@ -15,6 +15,7 @@
   <sheets>
     <sheet name="Chiller" sheetId="17" r:id="rId1"/>
     <sheet name="AirSourceHeatPump" sheetId="18" r:id="rId2"/>
+    <sheet name="AirSourceHeatPumpHeating" sheetId="34" r:id="rId28"/>
     <sheet name="入力シート(VRF_E+CoolingMode)" sheetId="16" r:id="rId3"/>
     <sheet name="入力シート(VRF_E+HeatingMode)" sheetId="22" r:id="rId4"/>
     <sheet name="boundary_dataset_c" sheetId="23" state="hidden" r:id="rId5"/>
@@ -9783,6 +9784,220 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F11"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rated hot water outlet temp.['C]</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>rated hot water inlet temp.['C]</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>rated hot water flow[m3/min]</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>rated power[kW]</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>hot water pressure loss coefficient[kPa/(m3/min)^2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>45</v>
+      </c>
+      <c r="B2">
+        <v>40</v>
+      </c>
+      <c r="C2">
+        <v>0.215</v>
+      </c>
+      <c r="D2">
+        <v>25</v>
+      </c>
+      <c r="E2">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>outdoor air temp.-load factor</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>0.2</v>
+      </c>
+      <c r="C4">
+        <v>0.4</v>
+      </c>
+      <c r="D4">
+        <v>0.6</v>
+      </c>
+      <c r="E4">
+        <v>0.8</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>-15</v>
+      </c>
+      <c r="B5">
+        <v>1.9</v>
+      </c>
+      <c r="C5">
+        <v>2.1</v>
+      </c>
+      <c r="D5">
+        <v>2.2</v>
+      </c>
+      <c r="E5">
+        <v>2.1</v>
+      </c>
+      <c r="F5">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>-10</v>
+      </c>
+      <c r="B6">
+        <v>2.2</v>
+      </c>
+      <c r="C6">
+        <v>2.4</v>
+      </c>
+      <c r="D6">
+        <v>2.5</v>
+      </c>
+      <c r="E6">
+        <v>2.4</v>
+      </c>
+      <c r="F6">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>-5</v>
+      </c>
+      <c r="B7">
+        <v>2.5</v>
+      </c>
+      <c r="C7">
+        <v>2.8</v>
+      </c>
+      <c r="D7">
+        <v>2.9</v>
+      </c>
+      <c r="E7">
+        <v>2.8</v>
+      </c>
+      <c r="F7">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>0</v>
+      </c>
+      <c r="B8">
+        <v>2.8</v>
+      </c>
+      <c r="C8">
+        <v>3.1</v>
+      </c>
+      <c r="D8">
+        <v>3.2</v>
+      </c>
+      <c r="E8">
+        <v>3.1</v>
+      </c>
+      <c r="F8">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>3.2</v>
+      </c>
+      <c r="C9">
+        <v>3.5</v>
+      </c>
+      <c r="D9">
+        <v>3.6</v>
+      </c>
+      <c r="E9">
+        <v>3.5</v>
+      </c>
+      <c r="F9">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>3.6</v>
+      </c>
+      <c r="C10">
+        <v>4</v>
+      </c>
+      <c r="D10">
+        <v>4.1</v>
+      </c>
+      <c r="E10">
+        <v>3.9</v>
+      </c>
+      <c r="F10">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <v>4</v>
+      </c>
+      <c r="C11">
+        <v>4.4</v>
+      </c>
+      <c r="D11">
+        <v>4.5</v>
+      </c>
+      <c r="E11">
+        <v>4.3</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C772E0E-249D-4F58-8692-A85D67698FF4}">
   <dimension ref="A1:Q76"/>

</xml_diff>

<commit_message>
Update AirSourceHeatPumpHeating (align rated power with COP table, unify sheet header format, bump version)
</commit_message>
<xml_diff>
--- a/equipment_spec.xlsx
+++ b/equipment_spec.xlsx
@@ -9791,27 +9791,27 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>rated hot water outlet temp.['C]</t>
+          <t>rated hot water outlet temp. ['C]</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>rated hot water inlet temp.['C]</t>
+          <t>rated hot water inlet temp. ['C]</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>rated hot water flow[m3/min]</t>
+          <t>rated hot water flow [m3/min]</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>rated power[kW]</t>
+          <t>rated power [kW]</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>hot water pressure loss coefficient[kPa/(m3/min)^2]</t>
+          <t>hot water pressure loss coefficient [kPa/(m3/min)^2]</t>
         </is>
       </c>
     </row>
@@ -9826,7 +9826,7 @@
         <v>0.215</v>
       </c>
       <c r="D2">
-        <v>25</v>
+        <v>22.321180555555557</v>
       </c>
       <c r="E2">
         <v>13.9</v>

</xml_diff>